<commit_message>
Major edits to change naming conventions of files and classes
</commit_message>
<xml_diff>
--- a/Data/2009_F033_CO_RSIS/2009_F033_CO_RSIS_RS.xlsx
+++ b/Data/2009_F033_CO_RSIS/2009_F033_CO_RSIS_RS.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\2009_F033_CO_RSIS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF98A4BD-FCB1-42D3-B298-60818AC0FCAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDC421C6-170C-4AF1-97BD-AA2915291667}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1575" yWindow="-27240" windowWidth="17910" windowHeight="17295" xr2:uid="{52B5C46F-C456-4503-98D2-245CB4BB11E3}"/>
+    <workbookView xWindow="-1755" yWindow="-27630" windowWidth="16140" windowHeight="16155" xr2:uid="{52B5C46F-C456-4503-98D2-245CB4BB11E3}"/>
   </bookViews>
   <sheets>
     <sheet name="HANDVI" sheetId="4" r:id="rId1"/>
-    <sheet name="Zones2NDVI" sheetId="3" r:id="rId2"/>
-    <sheet name="PlotsNDVI" sheetId="5" r:id="rId3"/>
+    <sheet name="ZoneNDVI" sheetId="3" r:id="rId2"/>
+    <sheet name="PlotNDVI" sheetId="5" r:id="rId3"/>
     <sheet name="HALST" sheetId="7" r:id="rId4"/>
-    <sheet name="Zones2LST" sheetId="6" r:id="rId5"/>
-    <sheet name="PlotsLST" sheetId="8" r:id="rId6"/>
+    <sheet name="ZoneLST" sheetId="6" r:id="rId5"/>
+    <sheet name="PlotLST" sheetId="8" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>